<commit_message>
build: rebuild dev jar for latest pull updates
</commit_message>
<xml_diff>
--- a/docs/202606타계정입고.xlsx
+++ b/docs/202606타계정입고.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\dwisCOST\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94F79F21-E149-45B6-A6E5-066786893490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D01C84-EFAF-4A86-96B1-FB4203B71C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{3640CD42-FD1E-42CB-9819-B8E00CC7FD25}"/>
+    <workbookView xWindow="-878" yWindow="990" windowWidth="21826" windowHeight="11437" xr2:uid="{3640CD42-FD1E-42CB-9819-B8E00CC7FD25}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="59">
   <si>
     <t>YYYYMM</t>
   </si>
@@ -117,9 +117,6 @@
   </si>
   <si>
     <t>MODEL_TYPE</t>
-  </si>
-  <si>
-    <t>STOCK</t>
   </si>
   <si>
     <t>BOH</t>
@@ -208,6 +205,22 @@
   </si>
   <si>
     <t>&lt;DOI_STOCK : 창고수량&gt;</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>WH0020 - Rework 완제품 창고</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>STOCK</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>WH0006-출하창고</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>* 수불의 out_month = (WH0006-출하창고.INPUT + WH0020 - Rework 완제품 창고.EOH)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -218,7 +231,7 @@
   <numFmts count="1">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -258,6 +271,15 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -460,7 +482,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -485,12 +507,6 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="41" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -520,6 +536,30 @@
     </xf>
     <xf numFmtId="41" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -856,7 +896,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9C513F7-B1A0-4833-BD67-F1C63BCD90BE}">
-  <dimension ref="A1:AP16"/>
+  <dimension ref="A1:AP21"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="8.6875" bestFit="1" customWidth="1"/>
@@ -896,135 +936,135 @@
   <sheetData>
     <row r="1" spans="1:42" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" t="s">
         <v>54</v>
-      </c>
-      <c r="P1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:42" x14ac:dyDescent="0.6">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="A2" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="M2" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="21" t="s">
         <v>13</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="Q2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="R2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="S2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="T2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="U2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="V2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="V2" s="6" t="s">
+      <c r="W2" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="W2" s="16" t="s">
+      <c r="X2" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="X2" s="7" t="s">
+      <c r="Y2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="Y2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="Z2" s="3" t="s">
+      <c r="AA2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="AA2" s="3" t="s">
+      <c r="AB2" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="AB2" s="3" t="s">
+      <c r="AC2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AD2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="AD2" s="3" t="s">
+      <c r="AE2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AE2" s="1" t="s">
+      <c r="AF2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AF2" s="1" t="s">
+      <c r="AG2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AG2" s="1" t="s">
+      <c r="AH2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AH2" s="1" t="s">
+      <c r="AI2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AI2" s="1" t="s">
+      <c r="AJ2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AJ2" s="1" t="s">
+      <c r="AK2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AK2" s="1" t="s">
+      <c r="AL2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AL2" s="1" t="s">
+      <c r="AM2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AM2" s="1" t="s">
+      <c r="AN2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AN2" s="1" t="s">
+      <c r="AO2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AO2" s="1" t="s">
+      <c r="AP2" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="AP2" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.6">
@@ -1058,10 +1098,10 @@
       <c r="J3" s="6">
         <v>19267</v>
       </c>
-      <c r="K3" s="10">
+      <c r="K3" s="8">
         <v>270323</v>
       </c>
-      <c r="L3" s="11">
+      <c r="L3" s="9">
         <v>270323</v>
       </c>
       <c r="M3" s="7">
@@ -1074,7 +1114,7 @@
         <v>17</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="R3" s="3">
         <v>387259</v>
@@ -1091,7 +1131,7 @@
       <c r="V3" s="6">
         <v>0</v>
       </c>
-      <c r="W3" s="17">
+      <c r="W3" s="15">
         <v>0</v>
       </c>
       <c r="X3" s="7">
@@ -1162,15 +1202,15 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="6"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="11"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="9"/>
       <c r="M4" s="7"/>
       <c r="N4" s="3"/>
       <c r="P4" s="5" t="s">
         <v>17</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R4" s="4">
         <v>0</v>
@@ -1184,13 +1224,13 @@
       <c r="U4" s="4">
         <v>8156</v>
       </c>
-      <c r="V4" s="14">
-        <v>0</v>
-      </c>
-      <c r="W4" s="18">
+      <c r="V4" s="12">
+        <v>0</v>
+      </c>
+      <c r="W4" s="16">
         <v>270323</v>
       </c>
-      <c r="X4" s="15">
+      <c r="X4" s="13">
         <v>-260644</v>
       </c>
       <c r="Y4" s="4">
@@ -1279,10 +1319,10 @@
       <c r="J5" s="6">
         <v>80</v>
       </c>
-      <c r="K5" s="10">
+      <c r="K5" s="8">
         <v>97</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="9">
         <v>97</v>
       </c>
       <c r="M5" s="7">
@@ -1295,7 +1335,7 @@
         <v>19</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R5" s="3">
         <v>0</v>
@@ -1312,7 +1352,7 @@
       <c r="V5" s="6">
         <v>0</v>
       </c>
-      <c r="W5" s="17">
+      <c r="W5" s="15">
         <v>0</v>
       </c>
       <c r="X5" s="7">
@@ -1383,15 +1423,15 @@
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="6"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="11"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="9"/>
       <c r="M6" s="7"/>
       <c r="N6" s="3"/>
       <c r="P6" s="5" t="s">
         <v>19</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="R6" s="4">
         <v>0</v>
@@ -1405,13 +1445,13 @@
       <c r="U6" s="4">
         <v>27</v>
       </c>
-      <c r="V6" s="14">
-        <v>0</v>
-      </c>
-      <c r="W6" s="18">
+      <c r="V6" s="12">
+        <v>0</v>
+      </c>
+      <c r="W6" s="16">
         <v>97</v>
       </c>
-      <c r="X6" s="15">
+      <c r="X6" s="13">
         <v>-70</v>
       </c>
       <c r="Y6" s="4">
@@ -1500,10 +1540,10 @@
       <c r="J7" s="6">
         <v>210</v>
       </c>
-      <c r="K7" s="10">
+      <c r="K7" s="8">
         <v>4429</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="9">
         <v>4429</v>
       </c>
       <c r="M7" s="7">
@@ -1516,7 +1556,7 @@
         <v>20</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R7" s="3">
         <v>450</v>
@@ -1533,7 +1573,7 @@
       <c r="V7" s="6">
         <v>0</v>
       </c>
-      <c r="W7" s="17">
+      <c r="W7" s="15">
         <v>0</v>
       </c>
       <c r="X7" s="7">
@@ -1604,15 +1644,15 @@
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="6"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="11"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="9"/>
       <c r="M8" s="7"/>
       <c r="N8" s="3"/>
       <c r="P8" s="5" t="s">
         <v>20</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R8" s="4">
         <v>0</v>
@@ -1626,13 +1666,13 @@
       <c r="U8" s="4">
         <v>182</v>
       </c>
-      <c r="V8" s="14">
-        <v>0</v>
-      </c>
-      <c r="W8" s="18">
+      <c r="V8" s="12">
+        <v>0</v>
+      </c>
+      <c r="W8" s="16">
         <v>4429</v>
       </c>
-      <c r="X8" s="15">
+      <c r="X8" s="13">
         <v>-4247</v>
       </c>
       <c r="Y8" s="4">
@@ -1721,10 +1761,10 @@
       <c r="J9" s="6">
         <v>72</v>
       </c>
-      <c r="K9" s="10">
+      <c r="K9" s="8">
         <v>748</v>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="9">
         <v>748</v>
       </c>
       <c r="M9" s="7">
@@ -1737,7 +1777,7 @@
         <v>21</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R9" s="3">
         <v>0</v>
@@ -1754,7 +1794,7 @@
       <c r="V9" s="6">
         <v>0</v>
       </c>
-      <c r="W9" s="17">
+      <c r="W9" s="15">
         <v>0</v>
       </c>
       <c r="X9" s="7">
@@ -1825,15 +1865,15 @@
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="6"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="11"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="9"/>
       <c r="M10" s="7"/>
       <c r="N10" s="3"/>
       <c r="P10" s="5" t="s">
         <v>21</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="R10" s="4">
         <v>0</v>
@@ -1847,13 +1887,13 @@
       <c r="U10" s="4">
         <v>47</v>
       </c>
-      <c r="V10" s="14">
-        <v>0</v>
-      </c>
-      <c r="W10" s="18">
+      <c r="V10" s="12">
+        <v>0</v>
+      </c>
+      <c r="W10" s="16">
         <v>748</v>
       </c>
-      <c r="X10" s="15">
+      <c r="X10" s="13">
         <v>-701</v>
       </c>
       <c r="Y10" s="4">
@@ -1942,10 +1982,10 @@
       <c r="J11" s="6">
         <v>66</v>
       </c>
-      <c r="K11" s="10">
+      <c r="K11" s="8">
         <v>462</v>
       </c>
-      <c r="L11" s="11">
+      <c r="L11" s="9">
         <v>462</v>
       </c>
       <c r="M11" s="7">
@@ -1958,7 +1998,7 @@
         <v>22</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R11" s="3">
         <v>0</v>
@@ -1975,7 +2015,7 @@
       <c r="V11" s="6">
         <v>0</v>
       </c>
-      <c r="W11" s="17">
+      <c r="W11" s="15">
         <v>0</v>
       </c>
       <c r="X11" s="7">
@@ -2046,15 +2086,15 @@
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="6"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="11"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="9"/>
       <c r="M12" s="7"/>
       <c r="N12" s="3"/>
       <c r="P12" s="5" t="s">
         <v>22</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="R12" s="4">
         <v>0</v>
@@ -2068,13 +2108,13 @@
       <c r="U12" s="4">
         <v>58</v>
       </c>
-      <c r="V12" s="14">
-        <v>0</v>
-      </c>
-      <c r="W12" s="18">
+      <c r="V12" s="12">
+        <v>0</v>
+      </c>
+      <c r="W12" s="16">
         <v>462</v>
       </c>
-      <c r="X12" s="15">
+      <c r="X12" s="13">
         <v>-404</v>
       </c>
       <c r="Y12" s="4">
@@ -2163,10 +2203,10 @@
       <c r="J13" s="6">
         <v>68</v>
       </c>
-      <c r="K13" s="10">
+      <c r="K13" s="8">
         <v>152</v>
       </c>
-      <c r="L13" s="11">
+      <c r="L13" s="9">
         <v>152</v>
       </c>
       <c r="M13" s="7">
@@ -2179,7 +2219,7 @@
         <v>23</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R13" s="3">
         <v>0</v>
@@ -2196,7 +2236,7 @@
       <c r="V13" s="6">
         <v>0</v>
       </c>
-      <c r="W13" s="17">
+      <c r="W13" s="15">
         <v>0</v>
       </c>
       <c r="X13" s="7">
@@ -2267,15 +2307,15 @@
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="6"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="11"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="9"/>
       <c r="M14" s="7"/>
       <c r="N14" s="3"/>
       <c r="P14" s="5" t="s">
         <v>23</v>
       </c>
       <c r="Q14" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="R14" s="4">
         <v>0</v>
@@ -2289,13 +2329,13 @@
       <c r="U14" s="4">
         <v>21</v>
       </c>
-      <c r="V14" s="14">
-        <v>0</v>
-      </c>
-      <c r="W14" s="18">
+      <c r="V14" s="12">
+        <v>0</v>
+      </c>
+      <c r="W14" s="16">
         <v>152</v>
       </c>
-      <c r="X14" s="15">
+      <c r="X14" s="13">
         <v>-131</v>
       </c>
       <c r="Y14" s="4">
@@ -2384,10 +2424,10 @@
       <c r="J15" s="6">
         <v>13577</v>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="10">
         <v>10275</v>
       </c>
-      <c r="L15" s="13">
+      <c r="L15" s="11">
         <v>10275</v>
       </c>
       <c r="M15" s="7">
@@ -2400,7 +2440,7 @@
         <v>24</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R15" s="3">
         <v>235145</v>
@@ -2417,7 +2457,7 @@
       <c r="V15" s="6">
         <v>0</v>
       </c>
-      <c r="W15" s="17">
+      <c r="W15" s="15">
         <v>0</v>
       </c>
       <c r="X15" s="7">
@@ -2483,7 +2523,7 @@
         <v>24</v>
       </c>
       <c r="Q16" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="R16" s="4">
         <v>0</v>
@@ -2497,13 +2537,13 @@
       <c r="U16" s="4">
         <v>275</v>
       </c>
-      <c r="V16" s="14">
-        <v>0</v>
-      </c>
-      <c r="W16" s="19">
+      <c r="V16" s="12">
+        <v>0</v>
+      </c>
+      <c r="W16" s="17">
         <v>10275</v>
       </c>
-      <c r="X16" s="15">
+      <c r="X16" s="13">
         <v>-9996</v>
       </c>
       <c r="Y16" s="4">
@@ -2559,6 +2599,23 @@
       </c>
       <c r="AP16" s="1">
         <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.6">
+      <c r="B17" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.6">
+      <c r="T19" s="1">
+        <f>I3-S3</f>
+        <v>8156</v>
+      </c>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.6">
+      <c r="T21" s="1">
+        <f>I3-T4</f>
+        <v>764323</v>
       </c>
     </row>
   </sheetData>

</xml_diff>